<commit_message>
Final PCB Submitted to PCBWay.
</commit_message>
<xml_diff>
--- a/electrical-hardware/Flight-Controller/V2/Flight-Controller/Deliverables/Bill of Materials-Flight-Controller.xlsx
+++ b/electrical-hardware/Flight-Controller/V2/Flight-Controller/Deliverables/Bill of Materials-Flight-Controller.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shadab\UBC-Rocket\thrust_vectoring_consolidated\electrical-hardware\Flight-Controller\V2\Flight-Controller\Project Outputs for Flight-Controller\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C0C9BF3-BAFF-4318-A3CD-290297642D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDE52CC1-BB57-4509-9F6F-A4098F490EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{F2C66D95-D626-412A-848A-A80716CD8D20}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{9B7452B6-9E4F-403C-94FB-ED8B11700AA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-Flight-Contro" sheetId="1" r:id="rId1"/>
@@ -1097,7 +1097,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEA5BCBA-AF1D-4C3C-9313-6980F1D60A11}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{763276FC-ECD6-4322-BBC4-6EBA9317B3C2}">
   <dimension ref="A1:E63"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>

</xml_diff>

<commit_message>
PCB Ready for JLCPCB Order.
</commit_message>
<xml_diff>
--- a/electrical-hardware/Flight-Controller/V2/Flight-Controller/Deliverables/Bill of Materials-Flight-Controller.xlsx
+++ b/electrical-hardware/Flight-Controller/V2/Flight-Controller/Deliverables/Bill of Materials-Flight-Controller.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shadab\UBC-Rocket\thrust_vectoring_consolidated\electrical-hardware\Flight-Controller\V2\Flight-Controller\Project Outputs for Flight-Controller\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDE52CC1-BB57-4509-9F6F-A4098F490EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B04C2DAD-BE9C-4BAC-B72B-943318541002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{9B7452B6-9E4F-403C-94FB-ED8B11700AA4}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{F11B27EB-C891-45A0-8C1F-469E6D002F04}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-Flight-Contro" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="278">
   <si>
     <t>Manu Part #</t>
   </si>
@@ -59,6 +59,9 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>LCSC Part #</t>
+  </si>
+  <si>
     <t>KMR231GLFS</t>
   </si>
   <si>
@@ -68,6 +71,9 @@
     <t>B1</t>
   </si>
   <si>
+    <t>C99271</t>
+  </si>
+  <si>
     <t>QMB-09B-05</t>
   </si>
   <si>
@@ -77,40 +83,52 @@
     <t>BZ1</t>
   </si>
   <si>
-    <t>CL21A226MAYNNNE</t>
+    <t>C161819</t>
+  </si>
+  <si>
+    <t>CL21A226MAQNNNE</t>
   </si>
   <si>
     <t>22uF ±20% 25V Ceramic Capacitor X5R 0805</t>
   </si>
   <si>
-    <t>C1, C42, C63, C64</t>
+    <t>C1, C42, C64, C65</t>
   </si>
   <si>
     <t>CAPC2012X145N</t>
   </si>
   <si>
+    <t>C45783</t>
+  </si>
+  <si>
     <t>CC0603KRX7R9BB104</t>
   </si>
   <si>
     <t>50V 100nF X7R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
   </si>
   <si>
-    <t>C2, C4, C5, C6, C7, C8, C9, C10, C11, C12, C13, C14, C15, C16, C17, C21, C22, C24, C26, C29, C30, C31, C32, C34, C37, C40, C43, C44, C47, C48, C50, C51, C52, C54, C55, C56, C57, C58, C59, C60</t>
+    <t>C2, C3, C5, C6, C7, C8, C9, C10, C11, C12, C13, C14, C15, C16, C17, C21, C22, C24, C26, C29, C30, C31, C32, C34, C37, C40, C44, C49, C50, C52, C53, C54, C56, C57, C58, C59, C60, C61, C62</t>
   </si>
   <si>
     <t>CAPC1608X90N</t>
   </si>
   <si>
-    <t>CC0603KRX7R9BB105</t>
+    <t>C14663</t>
+  </si>
+  <si>
+    <t>CL10A105KB8NNNC</t>
   </si>
   <si>
     <t>50V 1uF X7R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
   </si>
   <si>
-    <t>C3, C18, C25, C36, C49</t>
-  </si>
-  <si>
-    <t>CC0603KRX5R8BB225</t>
+    <t>C4, C18, C25, C36, C51</t>
+  </si>
+  <si>
+    <t>C15849</t>
+  </si>
+  <si>
+    <t>CL10A225KO8NNNC</t>
   </si>
   <si>
     <t>2.2 µF ±10% 25V Ceramic Capacitor X5R 0603 (1608 Metric)</t>
@@ -119,16 +137,22 @@
     <t>C19, C20, C35</t>
   </si>
   <si>
-    <t>CC0603KRX5R8BB475</t>
-  </si>
-  <si>
-    <t>4.7uF ±10% 25V Ceramic Capacitor X5R 0603</t>
+    <t>C23630</t>
+  </si>
+  <si>
+    <t>CL10A475KO8NNNC</t>
+  </si>
+  <si>
+    <t>16V 4.7uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
   </si>
   <si>
     <t>C23</t>
   </si>
   <si>
-    <t>CC0603FRNPO9BN120</t>
+    <t>C19666</t>
+  </si>
+  <si>
+    <t>CL10C120JB8NNNC</t>
   </si>
   <si>
     <t>12pF ±1% 50V Ceramic Capacitor NP0 0603</t>
@@ -137,31 +161,64 @@
     <t>C27, C28</t>
   </si>
   <si>
+    <t>C38523</t>
+  </si>
+  <si>
+    <t>0603B103K500NT</t>
+  </si>
+  <si>
+    <t>10nF ±10% 50V Ceramic Capacitor X7R 0603</t>
+  </si>
+  <si>
+    <t>C33, C39, C45</t>
+  </si>
+  <si>
+    <t>C57112</t>
+  </si>
+  <si>
+    <t>CL10A106KP8NNNC</t>
+  </si>
+  <si>
+    <t>10uF ±10% 10V Ceramic Capacitor X5R 0603</t>
+  </si>
+  <si>
+    <t>C38, C41, C43, C55</t>
+  </si>
+  <si>
+    <t>C19702</t>
+  </si>
+  <si>
+    <t>CL10C470JB8NNNC</t>
+  </si>
+  <si>
+    <t>47 pF ±5% 50V Ceramic Capacitor C0G, NP0 0603 (1608 Metric)</t>
+  </si>
+  <si>
+    <t>C46, C66</t>
+  </si>
+  <si>
+    <t>C1671</t>
+  </si>
+  <si>
     <t>CC0603KRX7R9BB103</t>
   </si>
   <si>
-    <t>10nF ±10% 50V Ceramic Capacitor X7R 0603</t>
-  </si>
-  <si>
-    <t>C33, C39, C46</t>
-  </si>
-  <si>
-    <t>CL21B106KAYQNNE</t>
-  </si>
-  <si>
-    <t>10uF ±10% 25V Ceramic Capacitor X7R 0805</t>
-  </si>
-  <si>
-    <t>C38, C41, C53, C61</t>
-  </si>
-  <si>
-    <t>CC0603JRNPO9BN470</t>
-  </si>
-  <si>
-    <t>47 pF ±5% 50V Ceramic Capacitor C0G, NP0 0603 (1608 Metric)</t>
-  </si>
-  <si>
-    <t>C45, C62</t>
+    <t>C47, C48</t>
+  </si>
+  <si>
+    <t>C100042</t>
+  </si>
+  <si>
+    <t>GRM21BR61H106KE43L</t>
+  </si>
+  <si>
+    <t>10uF 50V X5R ±10% 0805 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+  </si>
+  <si>
+    <t>C63</t>
+  </si>
+  <si>
+    <t>C440198</t>
   </si>
   <si>
     <t>1N5819HW-7-F</t>
@@ -176,6 +233,9 @@
     <t>SOD3716X125N</t>
   </si>
   <si>
+    <t>C82544</t>
+  </si>
+  <si>
     <t>BAT54XV2T1G</t>
   </si>
   <si>
@@ -188,6 +248,9 @@
     <t>SOD523</t>
   </si>
   <si>
+    <t>C81572</t>
+  </si>
+  <si>
     <t>BLM18AG601SN1D</t>
   </si>
   <si>
@@ -200,6 +263,9 @@
     <t>BLM18SP221SN1B</t>
   </si>
   <si>
+    <t>C19330</t>
+  </si>
+  <si>
     <t>BLM18SG330SN1D</t>
   </si>
   <si>
@@ -209,6 +275,9 @@
     <t>FB2</t>
   </si>
   <si>
+    <t>C576399</t>
+  </si>
+  <si>
     <t>STM32H745ZIT6</t>
   </si>
   <si>
@@ -221,6 +290,9 @@
     <t>QFP50P2200X2200X160-144N</t>
   </si>
   <si>
+    <t>C730193</t>
+  </si>
+  <si>
     <t>BMI088</t>
   </si>
   <si>
@@ -230,6 +302,9 @@
     <t>IC2</t>
   </si>
   <si>
+    <t>C194919</t>
+  </si>
+  <si>
     <t>MS561101BA03-50</t>
   </si>
   <si>
@@ -242,6 +317,9 @@
     <t>MSI-MS561101BA03-50-8_V</t>
   </si>
   <si>
+    <t>C15639</t>
+  </si>
+  <si>
     <t>ICM-40609-D</t>
   </si>
   <si>
@@ -254,6 +332,9 @@
     <t>LGA-24_L3.0-W3.0-P0.40-TL</t>
   </si>
   <si>
+    <t>C5360621</t>
+  </si>
+  <si>
     <t>MMC5983MA</t>
   </si>
   <si>
@@ -266,7 +347,10 @@
     <t>LGA-16_L3.0-W3.0-P0.50-BL_SQ</t>
   </si>
   <si>
-    <t>AZ1117CH-3.3TRG1</t>
+    <t>C404329</t>
+  </si>
+  <si>
+    <t>AMS1117-3.3</t>
   </si>
   <si>
     <t>70dB@(120Hz) 1.35A Fixed 3.3V Positive 10V SOT-223 Voltage Regulators - Linear, Low Drop Out (LDO) Regulators ROHS</t>
@@ -278,6 +362,9 @@
     <t>SOT230P700X180-4N</t>
   </si>
   <si>
+    <t>C6186</t>
+  </si>
+  <si>
     <t>ESDA6V1BC6</t>
   </si>
   <si>
@@ -290,6 +377,9 @@
     <t>SOT95P280X145-6N</t>
   </si>
   <si>
+    <t>C495220</t>
+  </si>
+  <si>
     <t>DP83848IVVX/NOPB</t>
   </si>
   <si>
@@ -302,13 +392,22 @@
     <t>QFP50P900X900X160-48N</t>
   </si>
   <si>
+    <t>C12082</t>
+  </si>
+  <si>
+    <t>TXS0104EPWR</t>
+  </si>
+  <si>
+    <t>4-Bit Bidirectional Voltage-Level Translator For Open-Drain and Push-Pull Applications</t>
+  </si>
+  <si>
+    <t>IC11</t>
+  </si>
+  <si>
     <t>TXB0104PWR</t>
   </si>
   <si>
-    <t>-40℃~+85℃ 1 1.2V~3.6V 1.65V~5.5V 100Mbps 4 Auto Direction Detection Bidirectional CMOS CMOS Tri-State TSSOP-14 Translators, Level Shifters ROHS</t>
-  </si>
-  <si>
-    <t>IC11</t>
+    <t>C44955</t>
   </si>
   <si>
     <t>SN74LVC2G241DCTR</t>
@@ -323,10 +422,13 @@
     <t>SOP65P400X130-8N</t>
   </si>
   <si>
+    <t>C2676069</t>
+  </si>
+  <si>
     <t>AP63300WU-7</t>
   </si>
   <si>
-    <t>Integrated Circuit</t>
+    <t>3.8V to 32V Input, 3A Low IQ Synchronous Buck Converter with Enhanced EMI Reduction</t>
   </si>
   <si>
     <t>IC13</t>
@@ -335,6 +437,9 @@
     <t>SOT95P280X90-6N</t>
   </si>
   <si>
+    <t>C2158012</t>
+  </si>
+  <si>
     <t>S4B-PH-K-S(LF)(SN)</t>
   </si>
   <si>
@@ -347,6 +452,9 @@
     <t>S4B-PH-K-S-_LF_SN</t>
   </si>
   <si>
+    <t>C157926</t>
+  </si>
+  <si>
     <t>S2B-PH-K-S(LF)(SN)</t>
   </si>
   <si>
@@ -359,6 +467,9 @@
     <t>S2B-PH-K-S_LF_SN</t>
   </si>
   <si>
+    <t>C173752</t>
+  </si>
+  <si>
     <t>S3B-PH-K-S(LF)(SN)</t>
   </si>
   <si>
@@ -371,6 +482,9 @@
     <t>S3B-PH-K-S-_LF_SN</t>
   </si>
   <si>
+    <t>C157929</t>
+  </si>
+  <si>
     <t>TF-01A</t>
   </si>
   <si>
@@ -383,6 +497,9 @@
     <t>TF-SMD_TF-01A</t>
   </si>
   <si>
+    <t>C41426929</t>
+  </si>
+  <si>
     <t>GT-USB-7010ASV</t>
   </si>
   <si>
@@ -395,6 +512,9 @@
     <t>USB-C-SMD_G-SWITCH_GT-USB-7010ASV</t>
   </si>
   <si>
+    <t>C2988369</t>
+  </si>
+  <si>
     <t>BWSMA-KWE-Z001</t>
   </si>
   <si>
@@ -407,6 +527,9 @@
     <t>SMA-TH_BWSMA-KWE-Z001</t>
   </si>
   <si>
+    <t>C496551</t>
+  </si>
+  <si>
     <t>HB-PH9-12727PB2GOB</t>
   </si>
   <si>
@@ -416,6 +539,9 @@
     <t>J13</t>
   </si>
   <si>
+    <t>C6332251</t>
+  </si>
+  <si>
     <t>XT60PW-F</t>
   </si>
   <si>
@@ -428,6 +554,9 @@
     <t>XT60PW-F_C428722</t>
   </si>
   <si>
+    <t>C428722</t>
+  </si>
+  <si>
     <t>DB125-2.54-4P-GN-S</t>
   </si>
   <si>
@@ -440,6 +569,9 @@
     <t>DB125-2_54-4P-GN</t>
   </si>
   <si>
+    <t>C918122</t>
+  </si>
+  <si>
     <t>LQG18HN27NJ00D</t>
   </si>
   <si>
@@ -449,7 +581,10 @@
     <t>L1</t>
   </si>
   <si>
-    <t>LQM18PH1R0MFRL</t>
+    <t>INDC1608X90N</t>
+  </si>
+  <si>
+    <t>C162550</t>
   </si>
   <si>
     <t>FXL0630-6R8-M</t>
@@ -461,46 +596,34 @@
     <t>L2</t>
   </si>
   <si>
-    <t>LTST-C170KRKT</t>
-  </si>
-  <si>
-    <t>Red 631nm LED Indication - Discrete 2V 0805 (2012 Metric)</t>
-  </si>
-  <si>
-    <t>LED1</t>
-  </si>
-  <si>
-    <t>LEDC2012X120N</t>
-  </si>
-  <si>
-    <t>LTST-C170GKT</t>
-  </si>
-  <si>
-    <t>Green 569nm LED Indication - Discrete 2.1V 0805 (2012 Metric)</t>
-  </si>
-  <si>
-    <t>LED2</t>
-  </si>
-  <si>
-    <t>SML-D12U8WT86C</t>
-  </si>
-  <si>
-    <t>Red LED Indication - Discrete 2.2V 0603</t>
-  </si>
-  <si>
-    <t>LED3</t>
+    <t>C167221</t>
+  </si>
+  <si>
+    <t>KT-0603R</t>
+  </si>
+  <si>
+    <t>-40℃~+85℃ 1.8V~2.4V 120° 20mA 300mcd 40mW 615nm~630nm 645nm Discrete Diode Red Water Clear 0603 LED Indication - Discrete ROHS</t>
+  </si>
+  <si>
+    <t>LED1, LED3</t>
   </si>
   <si>
     <t>LEDC1608X36N</t>
   </si>
   <si>
+    <t>C2286</t>
+  </si>
+  <si>
     <t>SML-E12P8WT86</t>
   </si>
   <si>
     <t>Green LED Indication - Discrete 2.2V 0603</t>
   </si>
   <si>
-    <t>LED4</t>
+    <t>LED2, LED4</t>
+  </si>
+  <si>
+    <t>C126319</t>
   </si>
   <si>
     <t>SML-D12Y1WT86</t>
@@ -512,18 +635,24 @@
     <t>LED5</t>
   </si>
   <si>
-    <t>2N7002,215</t>
+    <t>C253534</t>
+  </si>
+  <si>
+    <t>2N7002</t>
   </si>
   <si>
     <t>N-Channel 60V 300mA 830mW Surface Mount SOT-23</t>
   </si>
   <si>
-    <t>Q1, Q2, Q3</t>
+    <t>Q1, Q2, Q3, Q5, Q6, Q7, Q8</t>
   </si>
   <si>
     <t>SOT95P230X110-3N</t>
   </si>
   <si>
+    <t>C8545</t>
+  </si>
+  <si>
     <t>BSS8402DW-7-F</t>
   </si>
   <si>
@@ -536,100 +665,124 @@
     <t>SOT65P210X110-6N</t>
   </si>
   <si>
-    <t>IRLML6344TRPBF-ES</t>
-  </si>
-  <si>
-    <t>1 N-channel 1.4W 1.6V 170pF 25pF 30V 34mΩ@10V、50mΩ@4.5V 35pF 4.1nC@10V 4.3A N-Channel SOT-23 MOSFETs ROHS</t>
-  </si>
-  <si>
-    <t>Q5, Q6, Q7, Q8</t>
-  </si>
-  <si>
-    <t>RC0603JR-07330RL</t>
-  </si>
-  <si>
-    <t>330 Ohms ±5% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
-  </si>
-  <si>
-    <t>R1, R28, R29, R30, R61, R63, R65, R67</t>
+    <t>C156386</t>
+  </si>
+  <si>
+    <t>0603WAF4700T5E</t>
+  </si>
+  <si>
+    <t>-55℃~+155℃ 100mW 470Ω 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+  </si>
+  <si>
+    <t>R1, R29, R30, R31, R64, R66, R68</t>
+  </si>
+  <si>
+    <t>RESC1608X90N</t>
+  </si>
+  <si>
+    <t>C23179</t>
+  </si>
+  <si>
+    <t>0603WAF0000T5E</t>
+  </si>
+  <si>
+    <t>0Ω 100mW 75V Thick Film Resistor ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
+  </si>
+  <si>
+    <t>R2, R27, R28</t>
+  </si>
+  <si>
+    <t>C21189</t>
+  </si>
+  <si>
+    <t>0603WAF1002T5E</t>
+  </si>
+  <si>
+    <t>100mW Thick Film Resistor 75V ±100ppm/℃ ±1% 10kΩ 0603 Chip Resistor - Surface Mount ROHS</t>
+  </si>
+  <si>
+    <t>R3, R9, R10, R11, R12, R13, R14, R15, R16, R17, R18, R19, R20, R21, R22, R23, R48, R53, R54, R55, R56, R59, R61, R63, R65, R67, R69</t>
+  </si>
+  <si>
+    <t>C25804</t>
+  </si>
+  <si>
+    <t>0603WAF1001T5E</t>
+  </si>
+  <si>
+    <t>100mW 1kΩ 75V Thick Film Resistor ±100ppm/℃ ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
+  </si>
+  <si>
+    <t>R4, R6, R24, R60</t>
+  </si>
+  <si>
+    <t>C21190</t>
+  </si>
+  <si>
+    <t>0603WAF330JT5E</t>
+  </si>
+  <si>
+    <t>100mW 33Ω 75V Thick Film Resistor ±100ppm/℃ ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
+  </si>
+  <si>
+    <t>R5, R7, R8, R41, R44, R45, R49</t>
+  </si>
+  <si>
+    <t>C23140</t>
+  </si>
+  <si>
+    <t>RC0603FR-075K1L</t>
+  </si>
+  <si>
+    <t>100mW 5.1kΩ 75V Thick Film Resistor ±100ppm/℃ ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
+  </si>
+  <si>
+    <t>R25, R26</t>
   </si>
   <si>
     <t>RESC1608X55N</t>
   </si>
   <si>
-    <t>RC0603FR-070RL</t>
-  </si>
-  <si>
-    <t>0Ω 100mW 75V Thick Film Resistor ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
-  </si>
-  <si>
-    <t>R2, R27</t>
-  </si>
-  <si>
-    <t>RC0603FR-0710KL</t>
-  </si>
-  <si>
-    <t>100mW Thick Film Resistor 75V ±100ppm/℃ ±1% 10kΩ 0603 Chip Resistor - Surface Mount ROHS</t>
-  </si>
-  <si>
-    <t>R3, R9, R10, R11, R12, R13, R14, R15, R16, R17, R18, R19, R20, R21, R22, R23, R47, R52, R53, R54, R55, R58, R60, R64, R66, R68</t>
-  </si>
-  <si>
-    <t>RC0603FR-071KL</t>
-  </si>
-  <si>
-    <t>100mW 1kΩ 75V Thick Film Resistor ±100ppm/℃ ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
-  </si>
-  <si>
-    <t>R4, R6, R24, R59</t>
-  </si>
-  <si>
-    <t>RC0603FR-0733RL</t>
-  </si>
-  <si>
-    <t>100mW 33Ω 75V Thick Film Resistor ±100ppm/℃ ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
-  </si>
-  <si>
-    <t>R5, R7, R8, R40, R43, R44, R48</t>
-  </si>
-  <si>
-    <t>RC0603FR-075K1L</t>
-  </si>
-  <si>
-    <t>100mW 5.1kΩ 75V Thick Film Resistor ±100ppm/℃ ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
-  </si>
-  <si>
-    <t>R25, R26</t>
-  </si>
-  <si>
-    <t>RC0603FR-132K2L</t>
+    <t>C105580</t>
+  </si>
+  <si>
+    <t>0603WAF2201T5E</t>
   </si>
   <si>
     <t>2.2kΩ ±1% 100mW 0603 Thick Film Resistor</t>
   </si>
   <si>
-    <t>R31, R35, R36</t>
-  </si>
-  <si>
-    <t>R32, R33, R34, R37, R38, R39, R46</t>
-  </si>
-  <si>
-    <t>RC0603FR-0749R9L</t>
-  </si>
-  <si>
-    <t>100mW 49.9Ω 75V Thick Film Resistor ±100ppm/℃ ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
-  </si>
-  <si>
-    <t>R41, R42, R49, R50</t>
-  </si>
-  <si>
-    <t>RC0603FR-071K5L</t>
+    <t>R32, R36, R37</t>
+  </si>
+  <si>
+    <t>C4190</t>
+  </si>
+  <si>
+    <t>R33, R34, R35, R38, R39, R40, R47</t>
+  </si>
+  <si>
+    <t>0603WAF499JT5E</t>
+  </si>
+  <si>
+    <t>-55℃~+155℃ 100mW 49.9Ω 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+  </si>
+  <si>
+    <t>R42, R43, R50, R51</t>
+  </si>
+  <si>
+    <t>C23185</t>
+  </si>
+  <si>
+    <t>0603WAF1501T5E</t>
   </si>
   <si>
     <t>100mW 1.5kΩ 75V Thick Film Resistor ±100ppm/℃ ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
   </si>
   <si>
-    <t>R45</t>
+    <t>R46</t>
+  </si>
+  <si>
+    <t>C22843</t>
   </si>
   <si>
     <t>RC0603FR-074K87L</t>
@@ -638,36 +791,48 @@
     <t>4.87kΩ 100mW 75V Thick Film Resistor ±100ppm/℃ ±1% 0603 Chip Resistor - Surface Mount RoHS</t>
   </si>
   <si>
-    <t>R51</t>
-  </si>
-  <si>
-    <t>FRC0603F1583TS</t>
+    <t>R52</t>
+  </si>
+  <si>
+    <t>C137709</t>
+  </si>
+  <si>
+    <t>0603WAF1583T5E</t>
   </si>
   <si>
     <t>-55℃~+155℃ 100mW 158kΩ 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
   </si>
   <si>
-    <t>R56</t>
-  </si>
-  <si>
-    <t>RC0603FR-0730K1L</t>
-  </si>
-  <si>
-    <t>-55℃~+155℃ 100mW 30.1kΩ 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
-  </si>
-  <si>
     <t>R57</t>
   </si>
   <si>
-    <t>RC0603FR-0710RL</t>
-  </si>
-  <si>
-    <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±200ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+    <t>C22883</t>
+  </si>
+  <si>
+    <t>0603WAF3002T5E</t>
+  </si>
+  <si>
+    <t>-55℃~+155℃ 100mW 30kΩ 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+  </si>
+  <si>
+    <t>R58</t>
+  </si>
+  <si>
+    <t>C22984</t>
+  </si>
+  <si>
+    <t>0603WAF1200T5E</t>
+  </si>
+  <si>
+    <t>-55℃~+155℃ 100mW 120Ω 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
   </si>
   <si>
     <t>R62</t>
   </si>
   <si>
+    <t>C22787</t>
+  </si>
+  <si>
     <t>MAX-M10S-00B</t>
   </si>
   <si>
@@ -680,6 +845,9 @@
     <t>XCVR_MAX-M10S-00B</t>
   </si>
   <si>
+    <t>C4153167</t>
+  </si>
+  <si>
     <t>XC32M4-24.000-F12NJDTL</t>
   </si>
   <si>
@@ -692,6 +860,9 @@
     <t>CRYSTAL-SMD_4P-L3.2-W2.5-BL</t>
   </si>
   <si>
+    <t>C5122304</t>
+  </si>
+  <si>
     <t>SX3M50.000M20F30TNN</t>
   </si>
   <si>
@@ -702,6 +873,9 @@
   </si>
   <si>
     <t>SX3M50_000M20F30TNN</t>
+  </si>
+  <si>
+    <t>C2901592</t>
   </si>
 </sst>
 </file>
@@ -1097,17 +1271,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{763276FC-ECD6-4322-BBC4-6EBA9317B3C2}">
-  <dimension ref="A1:E63"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{977BB995-E390-4042-8D67-9A6633C2312C}">
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.53125" customWidth="1"/>
     <col min="2" max="3" width="18.53125" customWidth="1"/>
     <col min="4" max="4" width="15.53125" customWidth="1"/>
     <col min="5" max="5" width="18.53125" customWidth="1"/>
+    <col min="6" max="6" width="15.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1123,1059 +1298,1228 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="E2" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="E3" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F3" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E4" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F4" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E5" s="1">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E6" s="1">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F6" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="E7" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F7" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E8" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F8" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E9" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F9" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E10" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F10" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E11" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F11" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E12" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F12" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="E13" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+        <v>2</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="E14" s="1">
+        <v>1</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A16" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E16" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A15" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E15" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A16" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E16" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F16" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="E17" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F17" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="E18" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F18" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="E19" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F19" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="E20" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F20" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="E21" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F21" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="E22" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F22" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="E23" s="1">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A24" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E24" s="1">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A25" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E25" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A24" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E24" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A25" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E25" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F25" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="E26" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F26" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="E27" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F27" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>99</v>
+        <v>124</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="E28" s="1">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A29" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E29" s="1">
+        <v>1</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A30" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E30" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A29" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E29" s="1">
+      <c r="F30" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A31" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E31" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A30" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="E30" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A31" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E31" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F31" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>113</v>
+        <v>142</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>114</v>
+        <v>143</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>115</v>
+        <v>144</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>116</v>
+        <v>145</v>
       </c>
       <c r="E32" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F32" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>117</v>
+        <v>147</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="E33" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F33" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>122</v>
+        <v>153</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>123</v>
+        <v>154</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="E34" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F34" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
-        <v>124</v>
+        <v>157</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>125</v>
+        <v>158</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>126</v>
+        <v>159</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>127</v>
+        <v>160</v>
       </c>
       <c r="E35" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F35" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>128</v>
+        <v>162</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>130</v>
+        <v>164</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>131</v>
+        <v>162</v>
       </c>
       <c r="E36" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F36" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>132</v>
+        <v>166</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>133</v>
+        <v>167</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>134</v>
+        <v>168</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>135</v>
+        <v>169</v>
       </c>
       <c r="E37" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F37" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>136</v>
+        <v>171</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>137</v>
+        <v>172</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>138</v>
+        <v>173</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>136</v>
+        <v>174</v>
       </c>
       <c r="E38" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F38" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>139</v>
+        <v>176</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>140</v>
+        <v>177</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>141</v>
+        <v>178</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>142</v>
+        <v>179</v>
       </c>
       <c r="E39" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F39" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
-        <v>143</v>
+        <v>181</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>145</v>
+        <v>183</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>142</v>
+        <v>181</v>
       </c>
       <c r="E40" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F40" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>146</v>
+        <v>185</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>147</v>
+        <v>186</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>148</v>
+        <v>187</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="E41" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
+        <v>2</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>151</v>
+        <v>191</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>152</v>
+        <v>192</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="E42" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
+        <v>2</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>154</v>
+        <v>195</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>155</v>
+        <v>196</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="E43" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F43" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
-        <v>156</v>
+        <v>198</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>157</v>
+        <v>199</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>158</v>
+        <v>200</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>159</v>
+        <v>201</v>
       </c>
       <c r="E44" s="1">
+        <v>7</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A45" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E45" s="1">
+        <v>1</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A46" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E46" s="1">
+        <v>7</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A47" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E47" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A45" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="E45" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A46" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E46" s="1">
+      <c r="F47" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A48" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E48" s="1">
+        <v>27</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A49" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E49" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A47" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E47" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A48" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E48" s="1">
+      <c r="F49" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A50" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E50" s="1">
+        <v>7</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A51" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="E51" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A49" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E49" s="1">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A50" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E50" s="1">
+      <c r="F51" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A52" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E52" s="1">
+        <v>3</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A53" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E53" s="1">
+        <v>7</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A54" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E54" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A51" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E51" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A52" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E52" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A53" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E53" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A54" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E54" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F54" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
-        <v>190</v>
+        <v>243</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>191</v>
+        <v>244</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>192</v>
+        <v>245</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>170</v>
+        <v>211</v>
       </c>
       <c r="E55" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
-        <v>193</v>
+        <v>247</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>194</v>
+        <v>248</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>195</v>
+        <v>249</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>170</v>
+        <v>232</v>
       </c>
       <c r="E56" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F56" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
-        <v>196</v>
+        <v>251</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>197</v>
+        <v>252</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>198</v>
+        <v>253</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>170</v>
+        <v>211</v>
       </c>
       <c r="E57" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F57" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
-        <v>199</v>
+        <v>255</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>200</v>
+        <v>256</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>201</v>
+        <v>257</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>170</v>
+        <v>211</v>
       </c>
       <c r="E58" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F58" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
-        <v>202</v>
+        <v>259</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>203</v>
+        <v>260</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>204</v>
+        <v>261</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>170</v>
+        <v>211</v>
       </c>
       <c r="E59" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F59" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
-        <v>205</v>
+        <v>263</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>206</v>
+        <v>264</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>207</v>
+        <v>265</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>170</v>
+        <v>266</v>
       </c>
       <c r="E60" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F60" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
-        <v>208</v>
+        <v>268</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>209</v>
+        <v>269</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>210</v>
+        <v>270</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>211</v>
+        <v>271</v>
       </c>
       <c r="E61" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F61" s="2" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
-        <v>212</v>
+        <v>273</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>213</v>
+        <v>274</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>214</v>
+        <v>275</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>215</v>
+        <v>276</v>
       </c>
       <c r="E62" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A63" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="E63" s="1">
-        <v>1</v>
+      <c r="F62" s="2" t="s">
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final PCB Ordered from JLC.
</commit_message>
<xml_diff>
--- a/electrical-hardware/Flight-Controller/V2/Flight-Controller/Deliverables/Bill of Materials-Flight-Controller.xlsx
+++ b/electrical-hardware/Flight-Controller/V2/Flight-Controller/Deliverables/Bill of Materials-Flight-Controller.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shadab\UBC-Rocket\thrust_vectoring_consolidated\electrical-hardware\Flight-Controller\V2\Flight-Controller\Project Outputs for Flight-Controller\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B04C2DAD-BE9C-4BAC-B72B-943318541002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{31536E72-4B77-43B5-8F92-CDEC8AB5DC4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{F11B27EB-C891-45A0-8C1F-469E6D002F04}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{83643170-66B5-4795-9CEA-C49C626AD164}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-Flight-Contro" sheetId="1" r:id="rId1"/>
@@ -1271,7 +1271,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{977BB995-E390-4042-8D67-9A6633C2312C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84D46199-771D-4A21-A04D-AE3B6680F722}">
   <dimension ref="A1:F62"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>

</xml_diff>